<commit_message>
Lowered cap and started BOM
I lowered the filter cap to 2.2mF and started the BOM. I found a rectifier, rectifier capacitor, and diode. All that is left is the buck capacitor, MOSFET, and PCB stuff,
</commit_message>
<xml_diff>
--- a/Battery Charger Project/Excel/BOM/BOM V2.xlsx
+++ b/Battery Charger Project/Excel/BOM/BOM V2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Verrazano\Acedemic\Research\Battery-Charger\Battery Charger Project\Excel\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{981F17E4-5D91-4905-ADBB-B8048C88C8C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{199AE061-4643-4FFD-ACB7-A10735BD8D0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>item use</t>
   </si>
@@ -59,70 +59,67 @@
     <t>Total cost</t>
   </si>
   <si>
-    <t>Rectifier filter cap</t>
-  </si>
-  <si>
-    <t>CAP ALUM 2.7MF 20% 200V SNAP TH</t>
-  </si>
-  <si>
-    <t>B43544A2278M000</t>
-  </si>
-  <si>
-    <t>TDK</t>
-  </si>
-  <si>
-    <t>Buck capacitor</t>
-  </si>
-  <si>
-    <t>Würth Elektronik</t>
-  </si>
-  <si>
-    <t>Three phase rectifier</t>
-  </si>
-  <si>
     <t>link</t>
   </si>
   <si>
-    <t>Bridge Rectifiers Bridge, 3phase, DB, 200V, 15A, 150C, 350A</t>
-  </si>
-  <si>
-    <t>DB15-02</t>
-  </si>
-  <si>
-    <t>Diotec Semiconductor</t>
-  </si>
-  <si>
-    <t>https://www.mouser.com/en/ProductDetail/Diotec-Semiconductor/DB15-02?qs=OlC7AqGiEDmue9J3fser1A%3D%3D</t>
-  </si>
-  <si>
-    <t>CAP ALUM 10UF 20% 35V RADIAL TH</t>
-  </si>
-  <si>
-    <t>860020572003</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/w%C3%BCrth-elektronik/860020572003/5727172</t>
-  </si>
-  <si>
-    <t>Buck inductor</t>
-  </si>
-  <si>
     <t>LC200-0185</t>
   </si>
   <si>
     <t>437uH GE Inductor (Already in lab)</t>
   </si>
   <si>
-    <t>CAP ALUM 150UF 20% 200V RADIAL</t>
-  </si>
-  <si>
-    <t>P13520-ND</t>
-  </si>
-  <si>
     <t>DigiKey</t>
   </si>
   <si>
-    <t>https://www.digikey.com/en/products/detail/panasonic-industry/EEU-ED2D151/1086745</t>
+    <t>CAP ALUM 560UF 20% 200V SNAP TH</t>
+  </si>
+  <si>
+    <t>493-8516-ND</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/nichicon/LGW2D561MELA30/1966872</t>
+  </si>
+  <si>
+    <t>Bridge Rectifiers 200V 30A Power Diode Discretes-FRED i4-Pac</t>
+  </si>
+  <si>
+    <t>DPF30U200FC</t>
+  </si>
+  <si>
+    <t>MOUSER</t>
+  </si>
+  <si>
+    <t>https://www.mouser.com/en/ProductDetail/IXYS/DPF30U200FC?qs=rQFj71Wb1eWHztVyBgjseQ%3D%3D</t>
+  </si>
+  <si>
+    <t>Rectifier Capacitor</t>
+  </si>
+  <si>
+    <t>Buck Inductor</t>
+  </si>
+  <si>
+    <t>Three Phase Rectifier</t>
+  </si>
+  <si>
+    <t>Buck Capacitor</t>
+  </si>
+  <si>
+    <t>MOSFET</t>
+  </si>
+  <si>
+    <t>Diode</t>
+  </si>
+  <si>
+    <t>MBR10200_T0_00001</t>
+  </si>
+  <si>
+    <t>DIODE SCHOTTKY 200V 10A TO220AC</t>
+  </si>
+  <si>
+    <t>DigikKey</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/panjit-international-inc/MBR10200-T0-00001/15799461</t>
   </si>
 </sst>
 </file>
@@ -210,8 +207,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BE2F4241-DD34-429E-8619-5EC72E0D5702}" name="Table1" displayName="Table1" ref="A1:H5" totalsRowShown="0">
-  <autoFilter ref="A1:H5" xr:uid="{BE2F4241-DD34-429E-8619-5EC72E0D5702}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BE2F4241-DD34-429E-8619-5EC72E0D5702}" name="Table1" displayName="Table1" ref="A1:H7" totalsRowShown="0">
+  <autoFilter ref="A1:H7" xr:uid="{BE2F4241-DD34-429E-8619-5EC72E0D5702}"/>
   <tableColumns count="8">
     <tableColumn id="7" xr3:uid="{753B9BB0-B725-40B1-B016-495A15E17260}" name="item use"/>
     <tableColumn id="1" xr3:uid="{C3813DDA-4FC9-4A06-81E6-4B3D0E0DB3F4}" name="Item description"/>
@@ -495,7 +492,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="49.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="98.44140625" bestFit="1" customWidth="1"/>
@@ -518,7 +515,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
@@ -532,135 +529,146 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>23</v>
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="G2">
+        <v>5.25</v>
+      </c>
+      <c r="H2">
+        <f>Table1[[#This Row],[quantity]]*Table1[[#This Row],[unit price]]</f>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>2.33</v>
+        <v>20.09</v>
       </c>
       <c r="H3">
         <f>Table1[[#This Row],[quantity]]*Table1[[#This Row],[unit price]]</f>
-        <v>9.32</v>
+        <v>20.09</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>21</v>
+      </c>
       <c r="H5">
         <f>F5*G5</f>
         <v>0</v>
       </c>
     </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H6">
+        <f>F6*G6</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>1.29</v>
+      </c>
+      <c r="H7">
+        <f>F7*G7</f>
+        <v>1.29</v>
+      </c>
+    </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
       <c r="E9" s="2"/>
-      <c r="F9" s="2">
-        <v>3</v>
-      </c>
-      <c r="G9" s="2">
-        <v>24.05</v>
-      </c>
-      <c r="H9" s="2">
-        <f t="shared" ref="H9:H10" si="0">F9*G9</f>
-        <v>72.150000000000006</v>
-      </c>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" t="s">
-        <v>15</v>
-      </c>
-      <c r="C10" t="s">
-        <v>16</v>
-      </c>
-      <c r="D10" t="s">
-        <v>17</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F10">
-        <v>1</v>
-      </c>
-      <c r="G10" s="3">
-        <v>9.2799999999999994</v>
-      </c>
-      <c r="H10">
-        <f t="shared" si="0"/>
-        <v>9.2799999999999994</v>
-      </c>
+      <c r="E10" s="1"/>
+      <c r="G10" s="3"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F11" s="2">
-        <v>10</v>
-      </c>
-      <c r="G11" s="6">
-        <v>0.1</v>
-      </c>
-      <c r="H11" s="2">
-        <f>F11*G11</f>
-        <v>1</v>
-      </c>
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E10" r:id="rId1" xr:uid="{834A813A-2921-4DBA-951C-4D613A5B8572}"/>
-    <hyperlink ref="E11" r:id="rId2" xr:uid="{731E9BA3-84A5-4BF3-B19A-5D7D51647ABD}"/>
-    <hyperlink ref="E3" r:id="rId3" xr:uid="{E649B2B9-16DE-4CDD-9A8C-155AEF881E8C}"/>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{E649B2B9-16DE-4CDD-9A8C-155AEF881E8C}"/>
+    <hyperlink ref="E3" r:id="rId2" xr:uid="{1547E749-6240-43E7-A08B-467B1DD3808B}"/>
+    <hyperlink ref="E7" r:id="rId3" xr:uid="{DF8A8B79-7C2D-442E-AB3C-366F8EF73C57}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>